<commit_message>
Revisão geral: remove restos de rotas antigas e textos que contradiziam a ordem de Spirit
- Tyranny's Grip/Entangle/escudo fora da rota Chober
- Diagnóstico do Ato 4 com os supports certos
- Textos de esqueletos alinhados com a quantidade por fase
- Planilha regenerada com os mesmos dados

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
+++ b/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nível 1-100'!$A$3:$H$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Skills &amp; Supports'!$A$3:$J$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Quests'!$A$3:$F$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Tricks Pro'!$A$3:$D$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Tricks Pro'!$A$3:$D$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Uniques'!$A$3:$J$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1254,7 +1254,7 @@
       <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="104775" cy="419100"/>
+    <ext cx="333375" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="23" name="Image 23" descr="Picture"/>
@@ -1279,7 +1279,7 @@
       <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="333375" cy="419100"/>
+    <ext cx="419100" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="24" name="Image 24" descr="Picture"/>
@@ -1304,7 +1304,7 @@
       <row>27</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="419100"/>
+    <ext cx="276225" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="25" name="Image 25" descr="Picture"/>
@@ -1329,7 +1329,7 @@
       <row>28</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="276225" cy="419100"/>
+    <ext cx="419100" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="26" name="Image 26" descr="Picture"/>
@@ -1354,7 +1354,7 @@
       <row>29</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="419100"/>
+    <ext cx="419100" cy="247650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="27" name="Image 27" descr="Picture"/>
@@ -1379,7 +1379,7 @@
       <row>30</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="247650"/>
+    <ext cx="200025" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="28" name="Image 28" descr="Picture"/>
@@ -1404,7 +1404,7 @@
       <row>31</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="200025" cy="419100"/>
+    <ext cx="419100" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="29" name="Image 29" descr="Picture"/>
@@ -1429,7 +1429,7 @@
       <row>32</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="419100"/>
+    <ext cx="209550" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="30" name="Image 30" descr="Picture"/>
@@ -1454,7 +1454,7 @@
       <row>33</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="209550" cy="419100"/>
+    <ext cx="238125" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="31" name="Image 31" descr="Picture"/>
@@ -1479,7 +1479,7 @@
       <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="238125" cy="419100"/>
+    <ext cx="419100" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="32" name="Image 32" descr="Picture"/>
@@ -1504,7 +1504,7 @@
       <row>35</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="419100"/>
+    <ext cx="381000" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="33" name="Image 33" descr="Picture"/>
@@ -1529,7 +1529,7 @@
       <row>36</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="381000" cy="419100"/>
+    <ext cx="419100" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="34" name="Image 34" descr="Picture"/>
@@ -1554,7 +1554,7 @@
       <row>37</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="419100"/>
+    <ext cx="419100" cy="409575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="35" name="Image 35" descr="Picture"/>
@@ -1579,7 +1579,7 @@
       <row>38</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="419100" cy="409575"/>
+    <ext cx="104775" cy="419100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="36" name="Image 36" descr="Picture"/>
@@ -9043,12 +9043,12 @@
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>A troca: macaco + esqueletos</t>
+          <t>A troca: macaco + urso</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>5 tipos de esqueleto ativos · Muster no macaco · Lythara (+40 Spirit) · Resists no cap</t>
+          <t>2+ tipos de esqueleto (quantos couberem no Spirit) · Muster no macaco · Lythara (+40 Spirit) · Resists no cap</t>
         </is>
       </c>
       <c r="H25" s="16" t="n"/>
@@ -10463,7 +10463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10593,7 +10593,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Os 2 primeiros Skeletal Warriors são grátis</t>
+          <t>Rattling Sceptre já traz o esqueleto</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -10818,7 +10818,7 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Tyranny's Grip Runeforged sai ≈ 0,003 div e Chober Chaber Runeforged ≈ 0,04 div: mais barato do que juntar Verisium para fazer você mesmo.</t>
+          <t>Chober Chaber Runeforged sai ≈ 0,04 div: bem mais barato do que juntar Verisium para fazer você mesmo.</t>
         </is>
       </c>
     </row>
@@ -11060,7 +11060,7 @@
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Para achar companions no Hunting Grounds (Ato 1), tire o urso da ascendência e desative os companions — senão eles matam o beast antes do Tame Beast.</t>
+          <t>Quando for capturar um beast raro, desligue temporariamente os companions e o urso (Wild Protector) — senão eles matam o beast antes do Tame Beast pegar.</t>
         </is>
       </c>
     </row>
@@ -11086,7 +11086,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="34" customHeight="1">
+    <row r="30" ht="49" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
         <is>
           <t>Dano</t>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="D30" s="19" t="inlineStr">
         <is>
-          <t>Companions ganham 60% do dano da main-hand. Compare armas pelo dano mínimo–máximo, não pelo DPS: Tyranny's Grip tem attack speed reduzido e mesmo assim é a melhor opção barata.</t>
+          <t>Companions ganham 60% do dano da main-hand. Compare armas pelo dano mínimo–máximo por golpe, não pelo DPS: a Chober Chaber bate devagar, mas tem o maior dano por golpe e ainda dá +Minion Skills e Spirit.</t>
         </is>
       </c>
     </row>
@@ -11187,19 +11187,19 @@
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>Entangle é o seu botão principal</t>
+          <t>Fique perto (Presence)</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>No zoo, você não mata — você organiza. Entangle agrupa e prende os packs dentro do alcance do macaco e do urso. Use antes de cada pack grande.</t>
+          <t>Vários bônus (Shared Companion Damage, auras dos beasts) exigem companions na sua Presence. Não corra muito à frente do zoo em bosses.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Defesa</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
@@ -11209,12 +11209,12 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>Fique perto (Presence)</t>
+          <t>DoT é o que mata</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Vários bônus (Shared Companion Damage, auras dos beasts) exigem companions na sua Presence. Não corra muito à frente do zoo em bosses.</t>
+          <t>Evasion + Deflection seguram hits, não DoT. Leve Ruby (burn), Antidote (poison) e Staunching (bleed). Resists sempre no cap.</t>
         </is>
       </c>
     </row>
@@ -11226,43 +11226,43 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>Idolatry x runas de resist</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Cada Augment que não é Idol tira 4% de todas as resistências. Troque runas/soul cores de resist por Idols só depois de capar resists pelo gear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="49" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Economia</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
-        <is>
-          <t>DoT é o que mata</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>Evasion + Deflection seguram hits, não DoT. Leve Ruby (burn), Antidote (poison) e Staunching (bleed). Resists sempre no cap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="34" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
-        <is>
-          <t>Defesa</t>
-        </is>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
-      </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>Idolatry x runas de resist</t>
+          <t>Regex de vendor</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Cada Augment que não é Idol tira 4% de todas as resistências. Troque runas/soul cores de resist por Idols só depois de capar resists pelo gear.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="49" customHeight="1">
+          <t>Cole na busca do vendor para destacar upgrades: !regen|block|bow|mace|quarterstaff|armour:|accuracy|energy shield:""resi|\d+% i.+mov|ph.*da|\d l.+da|^\+.*ills$|^\+.*ion skills$|ck spe|o (all a|d)|evasion|spirit</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Economia</t>
@@ -11275,44 +11275,22 @@
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>Regex de vendor</t>
+          <t>Compre a Chober Chaber cedo</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
         <is>
-          <t>Cole na busca do vendor para destacar upgrades: !regen|block|bow|mace|quarterstaff|armour:|accuracy|energy shield:""resi|\d+% i.+mov|ph.*da|\d l.+da|^\+.*ills$|^\+.*ion skills$|ck spe|o (all a|d)|evasion|spirit</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="34" customHeight="1">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>Economia</t>
-        </is>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
-        <is>
-          <t>Fácil</t>
-        </is>
-      </c>
-      <c r="C39" s="18" t="inlineStr">
-        <is>
-          <t>Compre o Tyranny's Grip cedo</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>É um unique de nível 5 e costuma ser barato. Compre no Ato 4, guarde, e faça o Runeforge na Verisium Anvil quando pegar a Catha's Balance.</t>
+          <t>A Chober Chaber costuma custar poucos Exalts. Compre já Runeforged no Ato 3–4 e guarde: com a Catha's Balance ela vira a principal fonte de dano do zoo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D39"/>
+  <autoFilter ref="A3:D38"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:B39">
+  <conditionalFormatting sqref="B4:B38">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="5">
       <formula>"Fácil"</formula>
     </cfRule>
@@ -11419,7 +11397,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Supports errados: Muster · Armour Break II · Armour Demolisher II · Rage II. Suba o nível da gem Tame Beast.</t>
+          <t>Confira os supports do macaco: Feeding Frenzy II · Rage II · Rapid Attacks II · Heft (Muster só entra nos Interlúdios, quando tiver vários tipos de minion). Suba o nível da gem Tame Beast e use Sniper's Mark no boss.</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr"/>
@@ -11749,7 +11727,7 @@
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Tyranny's Grip / Trenchtimbre</t>
+          <t>Chober Chaber + Rattling Sceptre (ou Sylvan's Effigy)</t>
         </is>
       </c>
     </row>
@@ -12419,7 +12397,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="49" customHeight="1">
+    <row r="8" ht="64" customHeight="1">
       <c r="A8" s="23" t="n">
         <v>5</v>
       </c>
@@ -12430,12 +12408,12 @@
       </c>
       <c r="C8" s="19" t="inlineStr">
         <is>
-          <t>Ato 5: Frost Mage, Arsonist, Sniper, Reaver e Warrior ao mesmo tempo, sem supports de dano.</t>
+          <t>Mattjestic (Ato 5) usa Warrior, Arsonist, Sniper, Frost Mage e Reaver sem supports de dano — mas só com Spirit sobrando. Entre um por vez.</t>
         </is>
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Muster: +7% more dano para CADA tipo diferente de minion que revive. Cinco tipos de esqueleto baratos = +35% more dano no macaco, e ainda servem de alvo do Pain Offering.</t>
+          <t>Muster: +7% more dano para CADA tipo diferente de minion que revive. Cada tipo de esqueleto que couber no Spirit soma +7% no macaco e ainda serve de alvo do Pain Offering. 1 de cada tipo basta.</t>
         </is>
       </c>
       <c r="E8" s="42" t="inlineStr"/>
@@ -14528,7 +14506,7 @@
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>+100 Spirit num body de nível 1. É o maior ganho de Spirit da campanha: cabe mais um companion ou vários esqueletos.</t>
+          <t>+100 Spirit num body de nível 1. É o maior ganho de Spirit da campanha: cabe mais um companion (ou o beast de aura mais cedo).</t>
         </is>
       </c>
       <c r="I19" s="19" t="inlineStr">
@@ -14826,28 +14804,28 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="94" customHeight="1">
+    <row r="26" ht="64" customHeight="1">
       <c r="A26" s="19" t="inlineStr"/>
       <c r="B26" s="54" t="inlineStr">
         <is>
-          <t>Tyranny's Grip</t>
+          <t>Alpha's Howl</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>Main-hand</t>
+          <t>Capacete</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>Barato</t>
+          <t>Valor</t>
         </is>
       </c>
       <c r="E26" s="55" t="n">
-        <v>0.003</v>
+        <v>0.418</v>
       </c>
       <c r="F26" s="56" t="n">
-        <v>0.39</v>
+        <v>0.01</v>
       </c>
       <c r="G26" s="19" t="inlineStr">
         <is>
@@ -14856,59 +14834,10 @@
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>A arma barata padrão da Catha's Balance: +150–238% dano físico. Attack speed reduzido não importa, o companion ganha 60% do dano por golpe.</t>
+          <t>+100 Spirit e Presence em dobro (auras e bônus de Presence alcançam o zoo espalhado). Resolve o Spirit do modo barato.</t>
         </is>
       </c>
       <c r="I26" s="19" t="inlineStr">
-        <is>
-          <t>(150-192)% increased Physical Damage
-(10-15)% reduced Attack Speed
-+(15-30) to Strength
-Strikes deal Splash Damage
-Knocks Back Enemies on Hit
-Cannot use Projectile Attacks</t>
-        </is>
-      </c>
-      <c r="J26" s="19" t="inlineStr">
-        <is>
-          <t>Runeforged (nv 38) ≈ 0,003 div · Runemastered (nv 55) ≈ 0,41 div · Compre já Runeforged (sai mais barato que fazer). Runemastered adiciona 'Minions ganham 10% phys como lightning' e +20% dano de minion (bonded).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="64" customHeight="1">
-      <c r="A27" s="19" t="inlineStr"/>
-      <c r="B27" s="54" t="inlineStr">
-        <is>
-          <t>Alpha's Howl</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="inlineStr">
-        <is>
-          <t>Capacete</t>
-        </is>
-      </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="E27" s="55" t="n">
-        <v>0.418</v>
-      </c>
-      <c r="F27" s="56" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G27" s="19" t="inlineStr">
-        <is>
-          <t>Início do Atlas</t>
-        </is>
-      </c>
-      <c r="H27" s="19" t="inlineStr">
-        <is>
-          <t>+100 Spirit e Presence em dobro (auras e bônus de Presence alcançam o zoo espalhado). Resolve o Spirit do modo barato.</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
         <is>
           <t>(80-100)% increased Evasion Rating
 +100 to Spirit
@@ -14916,22 +14845,69 @@
 Presence Radius is doubled</t>
         </is>
       </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>≈ 0,42 div · Troca o +Minion Skills do capacete por Spirit: vale enquanto faltar reserva.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="56" customHeight="1">
+      <c r="A27" s="19" t="inlineStr"/>
+      <c r="B27" s="54" t="inlineStr">
+        <is>
+          <t>Undying Hate</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>Jewel</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="E27" s="55" t="n">
+        <v>0.529</v>
+      </c>
+      <c r="F27" s="56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>Início do Atlas</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>Timeless Jewel: conquista nós no raio com bônus Abyssal. Usado no mapping T1–10 do Mattjestic.</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Historic
+Conquered Attribute Passive Skills also grant +2 to Tribute</t>
+        </is>
+      </c>
       <c r="J27" s="19" t="inlineStr">
         <is>
-          <t>≈ 0,42 div · Troca o +Minion Skills do capacete por Spirit: vale enquanto faltar reserva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="56" customHeight="1">
+          <t xml:space="preserve"> · Opcional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="124" customHeight="1">
       <c r="A28" s="19" t="inlineStr"/>
       <c r="B28" s="54" t="inlineStr">
         <is>
-          <t>Undying Hate</t>
+          <t>Sylvan's Effigy</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Offhand</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
@@ -14940,12 +14916,10 @@
         </is>
       </c>
       <c r="E28" s="55" t="n">
-        <v>0.529</v>
-      </c>
-      <c r="F28" s="56" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.952</v>
+      </c>
+      <c r="F28" s="56" t="n">
+        <v>1</v>
       </c>
       <c r="G28" s="19" t="inlineStr">
         <is>
@@ -14954,55 +14928,10 @@
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>Timeless Jewel: conquista nós no raio com bônus Abyssal. Usado no mapping T1–10 do Mattjestic.</t>
+          <t>Companions ilimitados (tipos diferentes), Azmerian Wolf e Discipline de graça, +50–68% Spirit. Nesta liga custa ~1 div: não é luxo, é o primeiro grande objetivo do Atlas.</t>
         </is>
       </c>
       <c r="I28" s="19" t="inlineStr">
-        <is>
-          <t>Historic
-Conquered Attribute Passive Skills also grant +2 to Tribute</t>
-        </is>
-      </c>
-      <c r="J28" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> · Opcional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="124" customHeight="1">
-      <c r="A29" s="19" t="inlineStr"/>
-      <c r="B29" s="54" t="inlineStr">
-        <is>
-          <t>Sylvan's Effigy</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="inlineStr">
-        <is>
-          <t>Offhand</t>
-        </is>
-      </c>
-      <c r="D29" s="23" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="E29" s="55" t="n">
-        <v>0.952</v>
-      </c>
-      <c r="F29" s="56" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="19" t="inlineStr">
-        <is>
-          <t>Início do Atlas</t>
-        </is>
-      </c>
-      <c r="H29" s="19" t="inlineStr">
-        <is>
-          <t>Companions ilimitados (tipos diferentes), Azmerian Wolf e Discipline de graça, +50–68% Spirit. Nesta liga custa ~1 div: não é luxo, é o primeiro grande objetivo do Atlas.</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
         <is>
           <t>(50-68)% increased Spirit
 Allies in your Presence Regenerate (51.4-99.1) Life per second
@@ -15011,46 +14940,46 @@
 You can have any number of Companions of different types</t>
         </is>
       </c>
-      <c r="J29" s="19" t="inlineStr">
+      <c r="J28" s="19" t="inlineStr">
         <is>
           <t>≈ 0,95 div (4 mil à venda) · Coloque Primate Idol (+40% dano de aliados) e Rabbit Idol (+15% Spirit) nos sockets.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="94" customHeight="1">
-      <c r="A30" s="19" t="inlineStr"/>
-      <c r="B30" s="54" t="inlineStr">
+    <row r="29" ht="94" customHeight="1">
+      <c r="A29" s="19" t="inlineStr"/>
+      <c r="B29" s="54" t="inlineStr">
         <is>
           <t>Spiteful Floret</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
+      <c r="C29" s="19" t="inlineStr">
         <is>
           <t>Weapon set 2</t>
         </is>
       </c>
-      <c r="D30" s="23" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>Barato</t>
         </is>
       </c>
-      <c r="E30" s="55" t="n">
+      <c r="E29" s="55" t="n">
         <v>0.003</v>
       </c>
-      <c r="F30" s="56" t="n">
+      <c r="F29" s="56" t="n">
         <v>0.04</v>
       </c>
-      <c r="G30" s="19" t="inlineStr">
+      <c r="G29" s="19" t="inlineStr">
         <is>
           <t>T15+ (Effigy)</t>
         </is>
       </c>
-      <c r="H30" s="19" t="inlineStr">
+      <c r="H29" s="19" t="inlineStr">
         <is>
           <t>Fica no weapon set 2 só para conceder Sanguine Revelry (Remnants dão Rage e vida). Você não troca de set para lutar.</t>
         </is>
       </c>
-      <c r="I30" s="19" t="inlineStr">
+      <c r="I29" s="19" t="inlineStr">
         <is>
           <t>(60-90)% increased Physical Damage
 (6-10)% increased Attack Speed
@@ -15059,46 +14988,46 @@
 Every 5 Rage also grants 5% of Damage taken Recouped as Life</t>
         </is>
       </c>
-      <c r="J30" s="19" t="inlineStr">
+      <c r="J29" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve"> · Equipe no set 2 e ative Sanguine Revelry.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="154" customHeight="1">
-      <c r="A31" s="19" t="inlineStr"/>
-      <c r="B31" s="54" t="inlineStr">
+    <row r="30" ht="154" customHeight="1">
+      <c r="A30" s="19" t="inlineStr"/>
+      <c r="B30" s="54" t="inlineStr">
         <is>
           <t>Darkness Enthroned</t>
         </is>
       </c>
-      <c r="C31" s="19" t="inlineStr">
+      <c r="C30" s="19" t="inlineStr">
         <is>
           <t>Cinto</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D30" s="23" t="inlineStr">
         <is>
           <t>Barato</t>
         </is>
       </c>
-      <c r="E31" s="55" t="n">
+      <c r="E30" s="55" t="n">
         <v>0.014</v>
       </c>
-      <c r="F31" s="56" t="n">
+      <c r="F30" s="56" t="n">
         <v>0.02</v>
       </c>
-      <c r="G31" s="19" t="inlineStr">
+      <c r="G30" s="19" t="inlineStr">
         <is>
           <t>T15+ (Effigy)</t>
         </is>
       </c>
-      <c r="H31" s="19" t="inlineStr">
+      <c r="H30" s="19" t="inlineStr">
         <is>
           <t>Sockets de Augment tratados como Capacete/Escudo/Botas/Luvas com 50–99% mais efeito: mais Idols para a Idolatry.</t>
         </is>
       </c>
-      <c r="I31" s="19" t="inlineStr">
+      <c r="I30" s="19" t="inlineStr">
         <is>
           <t>(50-99)% increased effect of Socketed Augment Items
 This item gains bonuses from Socketed Items as though it was a Helmet
@@ -15107,46 +15036,46 @@
 This item gains bonuses from Socketed Items as though it was Gloves</t>
         </is>
       </c>
-      <c r="J31" s="19" t="inlineStr">
+      <c r="J30" s="19" t="inlineStr">
         <is>
           <t>≈ 0,014 div</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="94" customHeight="1">
-      <c r="A32" s="19" t="inlineStr"/>
-      <c r="B32" s="54" t="inlineStr">
+    <row r="31" ht="94" customHeight="1">
+      <c r="A31" s="19" t="inlineStr"/>
+      <c r="B31" s="54" t="inlineStr">
         <is>
           <t>The Hammer of Faith</t>
         </is>
       </c>
-      <c r="C32" s="19" t="inlineStr">
+      <c r="C31" s="19" t="inlineStr">
         <is>
           <t>Main-hand (2 mãos)</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="E32" s="55" t="n">
+      <c r="E31" s="55" t="n">
         <v>0.101</v>
       </c>
-      <c r="F32" s="56" t="n">
+      <c r="F31" s="56" t="n">
         <v>0.06</v>
       </c>
-      <c r="G32" s="19" t="inlineStr">
+      <c r="G31" s="19" t="inlineStr">
         <is>
           <t>T15+ (Effigy)</t>
         </is>
       </c>
-      <c r="H32" s="19" t="inlineStr">
+      <c r="H31" s="19" t="inlineStr">
         <is>
           <t>Giant Maul com 300–342% dano físico: muito dano por golpe para a Catha. Runeforged dá 30% phys como lightning e +60% dano de minion (bonded).</t>
         </is>
       </c>
-      <c r="I32" s="19" t="inlineStr">
+      <c r="I31" s="19" t="inlineStr">
         <is>
           <t>(300-339)% increased Physical Damage
 10% reduced Attack Speed
@@ -15155,9 +15084,54 @@
 Every 10 seconds, gain a random non-damaging Shrine buff for 20 seconds</t>
         </is>
       </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>≈ 0,10 div · Também exige Giant's Blood para usar com sceptre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="56" customHeight="1">
+      <c r="A32" s="19" t="inlineStr"/>
+      <c r="B32" s="54" t="inlineStr">
+        <is>
+          <t>Nascent Hope</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>Charm</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="E32" s="55" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="F32" s="56" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>T15+ (Effigy)</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>Thawing Charm que ganha cargas ao matar e inicia recarga de ES ao usar.</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr">
+        <is>
+          <t>(20-25)% Chance to gain a Charge when you kill an enemy
+Energy Shield Recharge starts on use</t>
+        </is>
+      </c>
       <c r="J32" s="19" t="inlineStr">
         <is>
-          <t>≈ 0,10 div · Também exige Giant's Blood para usar com sceptre.</t>
+          <t>≈ 0,11 div</t>
         </is>
       </c>
     </row>
@@ -15165,12 +15139,12 @@
       <c r="A33" s="19" t="inlineStr"/>
       <c r="B33" s="54" t="inlineStr">
         <is>
-          <t>Nascent Hope</t>
+          <t>Lavianga's Spirits</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Charm</t>
+          <t>Flask</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -15182,7 +15156,7 @@
         <v>0.106</v>
       </c>
       <c r="F33" s="56" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
@@ -15191,13 +15165,13 @@
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>Thawing Charm que ganha cargas ao matar e inicia recarga de ES ao usar.</t>
+          <t>Flask de mana com efeito constante: sustenta os Commands do Azmerian Wolf e marks, e combina com Mind Over Matter.</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>(20-25)% Chance to gain a Charge when you kill an enemy
-Energy Shield Recharge starts on use</t>
+          <t>This Flask cannot be Used but applies its Effect constantly
+(70-80)% reduced Amount Recovered</t>
         </is>
       </c>
       <c r="J33" s="19" t="inlineStr">
@@ -15206,16 +15180,16 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="56" customHeight="1">
+    <row r="34" ht="109" customHeight="1">
       <c r="A34" s="19" t="inlineStr"/>
       <c r="B34" s="54" t="inlineStr">
         <is>
-          <t>Lavianga's Spirits</t>
+          <t>Forgotten Warden</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Flask</t>
+          <t>Body Armour</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
@@ -15224,10 +15198,10 @@
         </is>
       </c>
       <c r="E34" s="55" t="n">
-        <v>0.106</v>
+        <v>0.209</v>
       </c>
       <c r="F34" s="56" t="n">
-        <v>0.25</v>
+        <v>0.8</v>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
@@ -15236,55 +15210,10 @@
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>Flask de mana com efeito constante: sustenta os Commands do Azmerian Wolf e marks, e combina com Mind Over Matter.</t>
+          <t>80% dos zoos usam. Companions +30–50% vida, Deflection, 10–15% do dano deflectido vai para os companions, e concede Spirit Vessel nível 16 (um companion a mais sem gastar gem).</t>
         </is>
       </c>
       <c r="I34" s="19" t="inlineStr">
-        <is>
-          <t>This Flask cannot be Used but applies its Effect constantly
-(70-80)% reduced Amount Recovered</t>
-        </is>
-      </c>
-      <c r="J34" s="19" t="inlineStr">
-        <is>
-          <t>≈ 0,11 div</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="109" customHeight="1">
-      <c r="A35" s="19" t="inlineStr"/>
-      <c r="B35" s="54" t="inlineStr">
-        <is>
-          <t>Forgotten Warden</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="inlineStr">
-        <is>
-          <t>Body Armour</t>
-        </is>
-      </c>
-      <c r="D35" s="23" t="inlineStr">
-        <is>
-          <t>Valor</t>
-        </is>
-      </c>
-      <c r="E35" s="55" t="n">
-        <v>0.209</v>
-      </c>
-      <c r="F35" s="56" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G35" s="19" t="inlineStr">
-        <is>
-          <t>T15+ (Effigy)</t>
-        </is>
-      </c>
-      <c r="H35" s="19" t="inlineStr">
-        <is>
-          <t>80% dos zoos usam. Companions +30–50% vida, Deflection, 10–15% do dano deflectido vai para os companions, e concede Spirit Vessel nível 16 (um companion a mais sem gastar gem).</t>
-        </is>
-      </c>
-      <c r="I35" s="19" t="inlineStr">
         <is>
           <t>+(70-100) to Deflection Rating per 50 missing Energy Shield
 (200-271)% increased Evasion and Energy Shield
@@ -15293,17 +15222,61 @@
 (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you</t>
         </is>
       </c>
+      <c r="J34" s="19" t="inlineStr">
+        <is>
+          <t>Base ≈ 0,21 div · Runemastered ≈ 5 div · Soquete Fox Idol (ativa bonded) e uma skill de Bear/Werewolf no Spirit Vessel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="64" customHeight="1">
+      <c r="A35" s="19" t="inlineStr"/>
+      <c r="B35" s="54" t="inlineStr">
+        <is>
+          <t>From Nothing</t>
+        </is>
+      </c>
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>Jewel</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="E35" s="55" t="n">
+        <v>0.212</v>
+      </c>
+      <c r="F35" s="56" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>T15+ (Effigy)</t>
+        </is>
+      </c>
+      <c r="H35" s="19" t="inlineStr">
+        <is>
+          <t>Aloca nós sem conexão: Vile Mending, Grip of Evil, Entropic Incarnation e o cluster de minion perto de Blackflame Covenant. É por isso que esses notables aparecem em 54–67% dos zoos top.</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Passives in Radius of (keystone) can be Allocated without being connected to your tree</t>
+        </is>
+      </c>
       <c r="J35" s="19" t="inlineStr">
         <is>
-          <t>Base ≈ 0,21 div · Runemastered ≈ 5 div · Soquete Fox Idol (ativa bonded) e uma skill de Bear/Werewolf no Spirit Vessel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="64" customHeight="1">
+          <t>≈ 0,21 div · Confira o keystone do raio no anúncio (precisa ser o que alcança os nós de minion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="56" customHeight="1">
       <c r="A36" s="19" t="inlineStr"/>
       <c r="B36" s="54" t="inlineStr">
         <is>
-          <t>From Nothing</t>
+          <t>Flesh Crucible</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
@@ -15317,10 +15290,12 @@
         </is>
       </c>
       <c r="E36" s="55" t="n">
-        <v>0.212</v>
-      </c>
-      <c r="F36" s="56" t="n">
-        <v>0.21</v>
+        <v>0.317</v>
+      </c>
+      <c r="F36" s="56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G36" s="19" t="inlineStr">
         <is>
@@ -15329,17 +15304,18 @@
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>Aloca nós sem conexão: Vile Mending, Grip of Evil, Entropic Incarnation e o cluster de minion perto de Blackflame Covenant. É por isso que esses notables aparecem em 54–67% dos zoos top.</t>
+          <t>Pode rolar Giant's Blood (entre outros keystones) com uma penalidade: alternativa ao Treefingers sem gastar slot de luva.</t>
         </is>
       </c>
       <c r="I36" s="19" t="inlineStr">
         <is>
-          <t>Passives in Radius of (keystone) can be Allocated without being connected to your tree</t>
+          <t>Concede 1 keystone aleatório (procure Giant's Blood)
+(10-20)% less de um atributo defensivo/ofensivo</t>
         </is>
       </c>
       <c r="J36" s="19" t="inlineStr">
         <is>
-          <t>≈ 0,21 div · Confira o keystone do raio no anúncio (precisa ser o que alcança os nós de minion).</t>
+          <t>≈ 0,32 div · Só compre a versão com Giant's Blood e penalidade leve (ex.: less mana).</t>
         </is>
       </c>
     </row>
@@ -15347,12 +15323,12 @@
       <c r="A37" s="19" t="inlineStr"/>
       <c r="B37" s="54" t="inlineStr">
         <is>
-          <t>Flesh Crucible</t>
+          <t>The Fall of the Axe</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Jewel</t>
+          <t>Charm</t>
         </is>
       </c>
       <c r="D37" s="23" t="inlineStr">
@@ -15361,12 +15337,10 @@
         </is>
       </c>
       <c r="E37" s="55" t="n">
-        <v>0.317</v>
-      </c>
-      <c r="F37" s="56" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.635</v>
+      </c>
+      <c r="F37" s="56" t="n">
+        <v>0.12</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
@@ -15375,43 +15349,42 @@
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>Pode rolar Giant's Blood (entre outros keystones) com uma penalidade: alternativa ao Treefingers sem gastar slot de luva.</t>
+          <t>Onslaught quando você é desacelerado: mais velocidade para acompanhar o zoo.</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Concede 1 keystone aleatório (procure Giant's Blood)
-(10-20)% less de um atributo defensivo/ofensivo</t>
+          <t>Grants Onslaught during effect</t>
         </is>
       </c>
       <c r="J37" s="19" t="inlineStr">
         <is>
-          <t>≈ 0,32 div · Só compre a versão com Giant's Blood e penalidade leve (ex.: less mana).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="56" customHeight="1">
+          <t>≈ 0,64 div</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="109" customHeight="1">
       <c r="A38" s="19" t="inlineStr"/>
       <c r="B38" s="54" t="inlineStr">
         <is>
-          <t>The Fall of the Axe</t>
+          <t>Controlled Metamorphosis</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Charm</t>
+          <t>Jewel</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>Valor</t>
+          <t>Luxo</t>
         </is>
       </c>
       <c r="E38" s="55" t="n">
-        <v>0.635</v>
+        <v>14.9</v>
       </c>
       <c r="F38" s="56" t="n">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="G38" s="19" t="inlineStr">
         <is>
@@ -15420,54 +15393,10 @@
       </c>
       <c r="H38" s="19" t="inlineStr">
         <is>
-          <t>Onslaught quando você é desacelerado: mais velocidade para acompanhar o zoo.</t>
+          <t>Aloca nós do anel médio-grande sem conexão (-5 a -20% resists). O Mattjestic usa para pegar nós de companion longe do caminho.</t>
         </is>
       </c>
       <c r="I38" s="19" t="inlineStr">
-        <is>
-          <t>Grants Onslaught during effect</t>
-        </is>
-      </c>
-      <c r="J38" s="19" t="inlineStr">
-        <is>
-          <t>≈ 0,64 div</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="109" customHeight="1">
-      <c r="A39" s="19" t="inlineStr"/>
-      <c r="B39" s="54" t="inlineStr">
-        <is>
-          <t>Controlled Metamorphosis</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="inlineStr">
-        <is>
-          <t>Jewel</t>
-        </is>
-      </c>
-      <c r="D39" s="23" t="inlineStr">
-        <is>
-          <t>Luxo</t>
-        </is>
-      </c>
-      <c r="E39" s="55" t="n">
-        <v>14.9</v>
-      </c>
-      <c r="F39" s="56" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G39" s="19" t="inlineStr">
-        <is>
-          <t>T15+ (Effigy)</t>
-        </is>
-      </c>
-      <c r="H39" s="19" t="inlineStr">
-        <is>
-          <t>Aloca nós do anel médio-grande sem conexão (-5 a -20% resists). O Mattjestic usa para pegar nós de companion longe do caminho.</t>
-        </is>
-      </c>
-      <c r="I39" s="19" t="inlineStr">
         <is>
           <t>Only affects Passives in Medium-Large Ring
 Only affects Passives in Massive Ring
@@ -15478,7 +15407,56 @@
 Only affects Passives in Very Small Ring</t>
         </is>
       </c>
-      <c r="J39" s="19" t="inlineStr"/>
+      <c r="J38" s="19" t="inlineStr"/>
+    </row>
+    <row r="39" ht="94" customHeight="1">
+      <c r="A39" s="19" t="inlineStr"/>
+      <c r="B39" s="54" t="inlineStr">
+        <is>
+          <t>Tyranny's Grip</t>
+        </is>
+      </c>
+      <c r="C39" s="19" t="inlineStr">
+        <is>
+          <t>Main-hand</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>Barato</t>
+        </is>
+      </c>
+      <c r="E39" s="55" t="n">
+        <v>0.003</v>
+      </c>
+      <c r="F39" s="56" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>Arbiter / Min-max</t>
+        </is>
+      </c>
+      <c r="H39" s="19" t="inlineStr">
+        <is>
+          <t>Arma barata popular da Catha's Balance em OUTRAS builds de zoo (spear de 1 mão). NÃO é usada nesta rota: aqui a Chober Chaber faz esse papel e ainda dá +Minion Skills e Spirit.</t>
+        </is>
+      </c>
+      <c r="I39" s="19" t="inlineStr">
+        <is>
+          <t>(150-192)% increased Physical Damage
+(10-15)% reduced Attack Speed
++(15-30) to Strength
+Strikes deal Splash Damage
+Knocks Back Enemies on Hit
+Cannot use Projectile Attacks</t>
+        </is>
+      </c>
+      <c r="J39" s="19" t="inlineStr">
+        <is>
+          <t>Runeforged (nv 38) ≈ 0,003 div · Runemastered (nv 55) ≈ 0,41 div · Só considere se não usar a rota Chober Chaber.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="56" customHeight="1">
       <c r="A40" s="19" t="inlineStr"/>
@@ -22691,17 +22669,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, Skeletal Warriors e Pain Offering.</t>
+          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, 1 Skeletal Warrior e Pain Offering.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>A troca: macaco + esqueletos</t>
+          <t>A troca: macaco + urso</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -22761,7 +22739,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Somar vários TIPOS de esqueleto (Frost Mage, Arsonist, Sniper, Reaver) só para o Muster: cada tipo diferente = +7% more dano no macaco. Vulnerability tira Armour.</t>
+          <t>Depois do Lythara (+40 Spirit), somar TIPOS de esqueleto para o Muster, um por vez e só enquanto couber no Spirit: cada tipo diferente = +7% more dano no macaco, e o 2º esqueleto libera o Danse Macabre. Vulnerability tira Armour.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -24544,7 +24522,7 @@
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, Skeletal Warriors e Pain Offering.</t>
+          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, 1 Skeletal Warrior e Pain Offering.</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -24564,7 +24542,7 @@
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I34" s="24">
@@ -24616,7 +24594,7 @@
       </c>
       <c r="H35" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I35" s="24">
@@ -24668,7 +24646,7 @@
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I36" s="24">
@@ -24720,7 +24698,7 @@
       </c>
       <c r="H37" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I37" s="24">
@@ -24772,7 +24750,7 @@
       </c>
       <c r="H38" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I38" s="24">
@@ -24824,7 +24802,7 @@
       </c>
       <c r="H39" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I39" s="24">
@@ -24876,7 +24854,7 @@
       </c>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I40" s="24">
@@ -24928,7 +24906,7 @@
       </c>
       <c r="H41" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I41" s="24">
@@ -24980,7 +24958,7 @@
       </c>
       <c r="H42" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I42" s="24">
@@ -25032,7 +25010,7 @@
       </c>
       <c r="H43" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I43" s="24">
@@ -25084,7 +25062,7 @@
       </c>
       <c r="H44" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I44" s="24">
@@ -25136,7 +25114,7 @@
       </c>
       <c r="H45" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I45" s="24">
@@ -25188,7 +25166,7 @@
       </c>
       <c r="H46" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I46" s="24">
@@ -25240,7 +25218,7 @@
       </c>
       <c r="H47" s="26" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I47" s="24">
@@ -25292,7 +25270,7 @@
       </c>
       <c r="H48" s="19" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="I48" s="24">
@@ -25844,7 +25822,7 @@
       </c>
       <c r="D59" s="26" t="inlineStr">
         <is>
-          <t>Somar vários TIPOS de esqueleto (Frost Mage, Arsonist, Sniper, Reaver) só para o Muster: cada tipo diferente = +7% more dano no macaco. Vulnerability tira Armour.</t>
+          <t>Depois do Lythara (+40 Spirit), somar TIPOS de esqueleto para o Muster, um por vez e só enquanto couber no Spirit: cada tipo diferente = +7% more dano no macaco, e o 2º esqueleto libera o Danse Macabre. Vulnerability tira Armour.</t>
         </is>
       </c>
       <c r="E59" s="26" t="inlineStr">
@@ -28591,7 +28569,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>ATO 3  ·  Nv 31–45  ·  A troca: macaco + esqueletos</t>
+          <t>ATO 3  ·  Nv 31–45  ·  A troca: macaco + urso</t>
         </is>
       </c>
       <c r="B31" s="14" t="n"/>
@@ -28608,7 +28586,7 @@
       </c>
       <c r="B32" s="29" t="inlineStr">
         <is>
-          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, Skeletal Warriors e Pain Offering.</t>
+          <t>Capturar o Mighty Silverfist com The Natural Order e trocar a build inteira para minions no mesmo dia: Twister sai, entram macaco, urso, 1 Skeletal Warrior e Pain Offering.</t>
         </is>
       </c>
       <c r="C32" s="10" t="n"/>
@@ -28624,7 +28602,7 @@
       </c>
       <c r="B33" s="29" t="inlineStr">
         <is>
-          <t>Mighty Silverfist (+ urso + esqueletos)</t>
+          <t>Mighty Silverfist (+ urso + 1 esqueleto)</t>
         </is>
       </c>
       <c r="C33" s="10" t="n"/>
@@ -28974,7 +28952,7 @@
       <c r="E60" s="14" t="n"/>
       <c r="F60" s="14" t="n"/>
     </row>
-    <row r="61" ht="19" customHeight="1">
+    <row r="61" ht="34" customHeight="1">
       <c r="A61" s="28" t="inlineStr">
         <is>
           <t>Objetivo</t>
@@ -28982,7 +28960,7 @@
       </c>
       <c r="B61" s="29" t="inlineStr">
         <is>
-          <t>Somar vários TIPOS de esqueleto (Frost Mage, Arsonist, Sniper, Reaver) só para o Muster: cada tipo diferente = +7% more dano no macaco. Vulnerability tira Armour.</t>
+          <t>Depois do Lythara (+40 Spirit), somar TIPOS de esqueleto para o Muster, um por vez e só enquanto couber no Spirit: cada tipo diferente = +7% more dano no macaco, e o 2º esqueleto libera o Danse Macabre. Vulnerability tira Armour.</t>
         </is>
       </c>
       <c r="C61" s="10" t="n"/>
@@ -29078,7 +29056,7 @@
       </c>
       <c r="B67" s="29" t="inlineStr">
         <is>
-          <t>5 tipos de esqueleto ativos · Muster no macaco · Lythara (+40 Spirit) · Resists no cap</t>
+          <t>2+ tipos de esqueleto (quantos couberem no Spirit) · Muster no macaco · Lythara (+40 Spirit) · Resists no cap</t>
         </is>
       </c>
       <c r="C67" s="10" t="n"/>
@@ -30527,7 +30505,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="34" customHeight="1">
+    <row r="19" ht="49" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Ato 3</t>
@@ -30555,7 +30533,7 @@
       </c>
       <c r="J19" s="19" t="inlineStr">
         <is>
-          <t>Bloqueia tudo enquanto segura. Precisa de escudo ou de um item que permita (substitui o Parry).</t>
+          <t>Só funciona com escudo ou buckler equipado. Com sceptre + maça (o set desta rota) ele não pode ser usado: deixe fora da barra se não tiver escudo.</t>
         </is>
       </c>
     </row>
@@ -31059,7 +31037,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
+    <row r="33" ht="49" customHeight="1">
       <c r="A33" s="26" t="inlineStr">
         <is>
           <t>Ato 4</t>
@@ -31087,7 +31065,7 @@
       </c>
       <c r="J33" s="26" t="inlineStr">
         <is>
-          <t>Bloqueio.</t>
+          <t>Só funciona com escudo ou buckler equipado. Com sceptre + maça (o set desta rota) ele não pode ser usado: deixe fora da barra se não tiver escudo.</t>
         </is>
       </c>
     </row>
@@ -32259,7 +32237,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="34" customHeight="1">
+    <row r="62" ht="64" customHeight="1">
       <c r="A62" s="19" t="inlineStr">
         <is>
           <t>T15+ (Effigy)</t>
@@ -32303,7 +32281,7 @@
       </c>
       <c r="J62" s="19" t="inlineStr">
         <is>
-          <t>Brutus' Brain: o espinho não pode ser destruído, então o buff nunca cai.</t>
+          <t>Brutus' Brain: o espinho não pode ser destruído, então o buff nunca cai. Danse Macabre só funciona com 2 esqueletos vivos: se você tiver só 1 Skeletal Cleric vivo, tire o Danse Macabre (os outros supports continuam valendo).</t>
         </is>
       </c>
     </row>
@@ -34218,7 +34196,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="49" customHeight="1">
+    <row r="4" ht="64" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Main-hand</t>
@@ -34226,12 +34204,12 @@
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>Campanha: spear rare. Ato 3: Trenchtimbre. Nv 65: Tyranny's Grip Runeforged (~0,003 div)</t>
+          <t>Atos 1–2: spear rare (Twister). Ato 3: Rattling Sceptre (main) + Trenchtimbre. Início do Atlas: Chober Chaber Runeforged (~0,04 div).</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>Tyranny's Grip Runemastered (~0,41 div) ou Trenchtimbre Runeforged</t>
+          <t>Chober Chaber Runeforged + Treefingers + The Vertex</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
@@ -34250,7 +34228,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="49" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>Offhand</t>
@@ -34258,7 +34236,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Campanha: escudo. Ato 3+: sceptre rare com Spirit</t>
+          <t>Atos 1–2: qualquer offhand. Ato 3+: Rattling Sceptre (base rare, traz Skeletal Warrior) com +Minion Skills</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
@@ -34346,7 +34324,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
+    <row r="8" ht="49" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Luvas</t>
@@ -34364,7 +34342,7 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Rare de Evasion/Deflection, Horror's Flight, ou Carved Majesty nas luvas</t>
+          <t>Treefingers até ter Giant's Blood na árvore; depois rare de Evasion/Deflection com vida e resist</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Aba Meu personagem com recomendações automáticas e limite real de companions
- Checklist: Spirit, keystones, ascendência, companions (beast + aura), esqueletos e itens
- Recomendações ao vivo (aba e painel lateral) com base no nível, modo e no que foi marcado
- Limite confirmado pelo texto do jogo: 1 base, 2 com Trusted Kinship/Yriel's Fostering, ilimitado com Sylvan's Effigy
- Ato 4 passa a ser 2 companions; 3º beast só com o Effigy

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
+++ b/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
@@ -29,7 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nível 1-100'!$A$3:$H$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Skills &amp; Supports'!$A$3:$J$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Quests'!$A$3:$F$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Tricks Pro'!$A$3:$D$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Tricks Pro'!$A$3:$D$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Uniques'!$A$3:$J$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>3 companions + chaos</t>
+          <t>2 companions + chaos</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
@@ -9102,7 +9102,7 @@
       </c>
       <c r="G24" s="19" t="inlineStr">
         <is>
-          <t>3 companions · Evergrasping Ring ×2 + Withering Presence · Testes de resistência do Ato 4 feitos</t>
+          <t>2 companions (macaco + aura) · Evergrasping Ring ×2 + Withering Presence · Testes de resistência do Ato 4 feitos</t>
         </is>
       </c>
       <c r="H24" s="16" t="n"/>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Giant's Blood + Chober + Effigy · Zekoa com Extra Crits/Haste · 3 aura bots · Forgotten Warden + Spirit Vessel</t>
+          <t>Giant's Blood + Chober + Effigy · Zekoa com Extra Crits/Haste · 3 aura bots (com Sylvan's Effigy) · Forgotten Warden + Spirit Vessel</t>
         </is>
       </c>
       <c r="H27" s="16" t="n"/>
@@ -10463,7 +10463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10522,237 +10522,237 @@
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Limite de companions</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Base: 1 companion. Trusted Kinship (keystone) ou Yriel's Fostering (body): 2 companions de TIPOS diferentes — não somam entre si. Sylvan's Effigy: qualquer número de tipos diferentes. O urso do Wild Protector não conta no limite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="79" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Captura</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Rota de aura bots do Mattjestic</t>
         </is>
       </c>
-      <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>1) Ato 4 Whakapanu Island: essence de crabs na praia (Quill/Coconut Crab ~25%) até achar Haste Aura. 2) Ato 5 Ashen Forest: Swarming Wisp (21%) com qualquer aura T1 exceto Haste. 3) Ato 2 Vastiri Outskirts: Crag Leaper (23,1%). Guarde auras T1 diferentes e substitua crabs duplicados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
-        <is>
-          <t>Captura</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="inlineStr">
-        <is>
-          <t>Fácil</t>
-        </is>
-      </c>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>Haste não aparece em beasts muito rápidos</t>
-        </is>
-      </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Beasts com a tag very_fast_movement (ex.: Crag Leaper) nunca rolam Haste Aura. Procure Haste em crabs.</t>
+          <t>Antes do Sylvan's Effigy só cabe 1 beast de aura (limite de 2 companions com Trusted Kinship). 1) Ato 4 Whakapanu Island: essence de crabs na praia (Quill/Coconut Crab ~25%) até achar Haste Aura. 2) Ato 5 Ashen Forest: Swarming Wisp (21%) com qualquer aura T1 exceto Haste. 3) Ato 2 Vastiri Outskirts: Crag Leaper (23,1%). Guarde auras T1 diferentes e substitua crabs duplicados. Os beasts extras entram quando você equipar o Effigy.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Dano</t>
+          <t>Captura</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Fácil</t>
         </is>
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Conte os tipos de minion para o Muster</t>
+          <t>Haste não aparece em beasts muito rápidos</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Urso, macaco, cada beast diferente, Azmerian Wolf, Wolf Pack, Spirit Vessel e cada tipo de esqueleto contam como um tipo. Cada um soma 7% more dano nos companions com Muster.</t>
+          <t>Beasts com a tag very_fast_movement (ex.: Crag Leaper) nunca rolam Haste Aura. Procure Haste em crabs.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Spirit</t>
+          <t>Dano</t>
         </is>
       </c>
       <c r="B7" s="23" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>Rattling Sceptre já traz o esqueleto</t>
+          <t>Conte os tipos de minion para o Muster</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>O Rattling Sceptre é uma base comum (não unique) que já traz a gem Skeletal Warrior. Um único esqueleto basta como alvo do Pain Offering até o Effigy; o segundo só quando sobrar Spirit.</t>
+          <t>Urso, macaco, cada beast diferente, Azmerian Wolf, Wolf Pack, Spirit Vessel e cada tipo de esqueleto contam como um tipo. Cada um soma 7% more dano nos companions com Muster.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
+          <t>Spirit</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Rattling Sceptre já traz o esqueleto</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>O Rattling Sceptre é uma base comum (não unique) que já traz a gem Skeletal Warrior. Um único esqueleto basta como alvo do Pain Offering até o Effigy; o segundo só quando sobrar Spirit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
           <t>Economia</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>The Vertex: confira a versão</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Só a versão com 'Equipment has no Attribute Requirements' libera a Chober Chaber com Giant's Blood. Filtre por esse mod no trade.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="49" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Dano</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>Pain Offering sem cair no boss</t>
-        </is>
-      </c>
-      <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>Brutus' Brain no Pain Offering deixa o espinho imune a dano, então o buff não some quando o boss acerta a área. Danse Macabre precisa de 2 esqueletos vivos: só coloque quando o Spirit permitir o 2º esqueleto (Interlúdios). Depois do Effigy, o Skeletal Cleric com Sacrificial Lamb II vira o alvo.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="49" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
         <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>Pain Offering sem cair no boss</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>Brutus' Brain no Pain Offering deixa o espinho imune a dano, então o buff não some quando o boss acerta a área. Danse Macabre precisa de 2 esqueletos vivos: só coloque quando o Spirit permitir o 2º esqueleto (Interlúdios). Depois do Effigy, o Skeletal Cleric com Sacrificial Lamb II vira o alvo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="49" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
           <t>Captura</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Como o Tame Beast funciona</t>
         </is>
       </c>
-      <c r="D10" s="19" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Use o Tame Beast num raro: ele fica envolto em wisps (Hinder) por ~8–12s. Mate enquanto os wisps estão nele para capturar. O beast guarda até 4 mods de monstro, então capture o que tem os mods que você quer.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="34" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>Silverfist</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Zekoa com 3+ mods</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Riverside ou Rupture + 1 Cruel Hegemony + 2 tablets raros com 'Unique Monsters have 1 additional Rare Modifier'. Ordem de mods: Extra Crits &gt; Hasted &gt; Extra Damage as Chaos/Physical &gt; Soul Eater.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="49" customHeight="1">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Silverfist</t>
-        </is>
-      </c>
-      <c r="B12" s="23" t="inlineStr">
-        <is>
-          <t>Avançado</t>
-        </is>
-      </c>
-      <c r="C12" s="18" t="inlineStr">
-        <is>
-          <t>Reroll de mods morrendo (softcore)</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>Com Doryani como Atlas Master e o nó Stitch the Flesh (revive extra), dá para morrer de propósito na luta e o boss volta com mods novos. Rituals perto de City biomes geram vários Zekoas no mesmo map.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="49" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
         <is>
+          <t>Silverfist</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Avançado</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Reroll de mods morrendo (softcore)</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>Com Doryani como Atlas Master e o nó Stitch the Flesh (revive extra), dá para morrer de propósito na luta e o boss volta com mods novos. Rituals perto de City biomes geram vários Zekoas no mesmo map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="49" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
           <t>Dano</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B14" s="23" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Giant's Blood + The Vertex</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>Treefingers dá Giant's Blood (maça 2 mãos + sceptre), mas triplica requisitos. The Vertex remove requisitos de gems (e, em algumas versões, do equipamento). Soul Core of Cholotl converte 40% para Dex.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>Spirit</t>
-        </is>
-      </c>
-      <c r="B14" s="23" t="inlineStr">
-        <is>
-          <t>Fácil</t>
-        </is>
-      </c>
-      <c r="C14" s="18" t="inlineStr">
-        <is>
-          <t>Idols no Sylvan's Effigy</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>Primate Idol (+40% dano de aliados) e Rabbit Idol (+15% Spirit) custam centavos. No capacete, Idol of Ralakesh dá +8% reservation efficiency de minions.</t>
         </is>
       </c>
     </row>
@@ -10769,19 +10769,19 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Alpha's Howl quando faltar Spirit</t>
+          <t>Idols no Sylvan's Effigy</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>+100 Spirit e Presence em dobro por ~0,4 div. Troque de volta por capacete com +Minion Skills quando o Spirit sobrar.</t>
+          <t>Primate Idol (+40% dano de aliados) e Rabbit Idol (+15% Spirit) custam centavos. No capacete, Idol of Ralakesh dá +8% reservation efficiency de minions.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="34" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
         <is>
-          <t>Dano</t>
+          <t>Spirit</t>
         </is>
       </c>
       <c r="B16" s="23" t="inlineStr">
@@ -10791,19 +10791,19 @@
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>Spirit Vessel do Forgotten Warden</t>
+          <t>Alpha's Howl quando faltar Spirit</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
-          <t>O body já concede Spirit Vessel nível 16. Soquete skills de Bear/Werewolf/Wyvern nele (ex.: Furious Slam): ganha 20% more dano por skill diferente.</t>
+          <t>+100 Spirit e Presence em dobro por ~0,4 div. Troque de volta por capacete com +Minion Skills quando o Spirit sobrar.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="34" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>Economia</t>
+          <t>Dano</t>
         </is>
       </c>
       <c r="B17" s="23" t="inlineStr">
@@ -10813,100 +10813,100 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Compre uniques já runeforged</t>
+          <t>Spirit Vessel do Forgotten Warden</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Chober Chaber Runeforged sai ≈ 0,04 div: bem mais barato do que juntar Verisium para fazer você mesmo.</t>
+          <t>O body já concede Spirit Vessel nível 16. Soquete skills de Bear/Werewolf/Wyvern nele (ex.: Furious Slam): ganha 20% more dano por skill diferente.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="19" t="inlineStr">
         <is>
-          <t>Defesa</t>
+          <t>Economia</t>
         </is>
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Fácil</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Mind Over Matter + Lavianga's Spirits</t>
+          <t>Compre uniques já runeforged</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>O flask de mana com efeito constante e a mana da Chober Chaber sustentam o MoM e os Commands do Azmerian Wolf.</t>
+          <t>Chober Chaber Runeforged sai ≈ 0,04 div: bem mais barato do que juntar Verisium para fazer você mesmo.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
         <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Mind Over Matter + Lavianga's Spirits</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>O flask de mana com efeito constante e a mana da Chober Chaber sustentam o MoM e os Commands do Azmerian Wolf.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
           <t>Forbidden Rites</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Ritual em toda área da campanha</t>
         </is>
       </c>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Nesta liga cada área da campanha tem um Ritual que dá currency de crafting e equipamento. Faça todos no Ato 1–2: é o jeito mais barato de achar spear e botas com Movement Speed sem gastar no trade.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="49" customHeight="1">
-      <c r="A20" s="19" t="inlineStr">
+    <row r="21" ht="49" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Forbidden Rites</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B21" s="23" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Cluster de Ritual em bosses = uniques</t>
         </is>
       </c>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="D21" s="19" t="inlineStr">
         <is>
           <t>Duas vezes por ato (e uma por interlúdio) aparecem clusters de Ritual Effigies em cima do boss da área. O boss derrotado se soma à próxima área do cluster; no fim você gasta Tribute em Unique Items. Guarde Tribute para isso e procure Meginord's Girdle ou Tyranny's Grip.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="19" t="inlineStr">
-        <is>
-          <t>Forbidden Rites</t>
-        </is>
-      </c>
-      <c r="B21" s="23" t="inlineStr">
-        <is>
-          <t>Fácil</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Trial of Chaos com pausa</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>No 0.5.5 dá para sair do Trial of Chaos e voltar depois na mesma sala, e cada sala tem baú de recompensa. Faça a 2ª Ascendência sem medo de perder a run se precisar parar para trade.</t>
         </is>
       </c>
     </row>
@@ -10918,61 +10918,61 @@
       </c>
       <c r="B22" s="23" t="inlineStr">
         <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Trial of Chaos com pausa</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>No 0.5.5 dá para sair do Trial of Chaos e voltar depois na mesma sala, e cada sala tem baú de recompensa. Faça a 2ª Ascendência sem medo de perder a run se precisar parar para trade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Forbidden Rites</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Trials 65+ dropam Exceptional</t>
         </is>
       </c>
-      <c r="D22" s="19" t="inlineStr">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Trial of Sekhemas e Trial of Chaos ganham bônus a partir de área 65 (mais raros, qualidade e itens Exceptional). Rodar a 3ª e 4ª Ascendência nesse nível paga o próprio custo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="49" customHeight="1">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>Forbidden Rites</t>
-        </is>
-      </c>
-      <c r="B23" s="23" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="inlineStr">
-        <is>
-          <t>Viridian Wildwood</t>
-        </is>
-      </c>
-      <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Sacred Blooms (recompensa de Ritual) adicionam o Viridian Wildwood a um grupo de maps. Siga as trilhas de Wisps: os monstros do map ficam mais fortes e mais recompensadores. Com o zoo em T15 isso é farm fácil.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="49" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Silverfist</t>
+          <t>Forbidden Rites</t>
         </is>
       </c>
       <c r="B24" s="23" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>Não mate o macaco cedo</t>
+          <t>Viridian Wildwood</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>Se chegar ao Jungle Ruins sem The Natural Order, não mate o Silverfist: siga, faça o Trial of Chaos e volte pelo waypoint para capturá-lo. Se já matou, sem pânico — ele é sempre o boss dos maps Riverside e Rupture.</t>
+          <t>Sacred Blooms (recompensa de Ritual) adicionam o Viridian Wildwood a um grupo de maps. Siga as trilhas de Wisps: os monstros do map ficam mais fortes e mais recompensadores. Com o zoo em T15 isso é farm fácil.</t>
         </is>
       </c>
     </row>
@@ -10984,61 +10984,61 @@
       </c>
       <c r="B25" s="23" t="inlineStr">
         <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Não mate o macaco cedo</t>
+        </is>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>Se chegar ao Jungle Ruins sem The Natural Order, não mate o Silverfist: siga, faça o Trial of Chaos e volte pelo waypoint para capturá-lo. Se já matou, sem pânico — ele é sempre o boss dos maps Riverside e Rupture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="49" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Silverfist</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="inlineStr">
+        <is>
           <t>Avançado</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>Silverfist com Extra Crits</t>
         </is>
       </c>
-      <c r="D25" s="19" t="inlineStr">
+      <c r="D26" s="19" t="inlineStr">
         <is>
           <t>Use tablets com 'Unique monsters have 1 additional modifier' + Cruel Hegemony (e o nó do Jado com 20% de chance de dobrar mods de tablet) em Riverside/Rupture. Mais mods = mais chances de Extra Crits. Não precisa de map alto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>Silverfist</t>
-        </is>
-      </c>
-      <c r="B26" s="23" t="inlineStr">
-        <is>
-          <t>Avançado</t>
-        </is>
-      </c>
-      <c r="C26" s="18" t="inlineStr">
-        <is>
-          <t>Rite of the Nameless</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Começar o Rite of the Nameless (Ritual) em Riverside/Rupture coloca o macaco no último ritual de cada map — mais tentativas de mods. É perigoso: vá com defesa em dia.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="34" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
         <is>
-          <t>Captura</t>
+          <t>Silverfist</t>
         </is>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Avançado</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>Pause no trade para ler mods</t>
+          <t>Rite of the Nameless</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Liga o atalho do Marketplace no botão do meio do mouse. Viu um beast raro? Aperta e o jogo pausa para você ler os mods com calma (não funciona em SSF).</t>
+          <t>Começar o Rite of the Nameless (Ritual) em Riverside/Rupture coloca o macaco no último ritual de cada map — mais tentativas de mods. É perigoso: vá com defesa em dia.</t>
         </is>
       </c>
     </row>
@@ -11055,12 +11055,12 @@
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>Caçar sem matar sem querer</t>
+          <t>Pause no trade para ler mods</t>
         </is>
       </c>
       <c r="D28" s="19" t="inlineStr">
         <is>
-          <t>Quando for capturar um beast raro, desligue temporariamente os companions e o urso (Wild Protector) — senão eles matam o beast antes do Tame Beast pegar.</t>
+          <t>Liga o atalho do Marketplace no botão do meio do mouse. Viu um beast raro? Aperta e o jogo pausa para você ler os mods com calma (não funciona em SSF).</t>
         </is>
       </c>
     </row>
@@ -11072,134 +11072,134 @@
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>Caçar sem matar sem querer</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Quando for capturar um beast raro, desligue temporariamente os companions e o urso (Wild Protector) — senão eles matam o beast antes do Tame Beast pegar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Captura</t>
+        </is>
+      </c>
+      <c r="B30" s="23" t="inlineStr">
+        <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Ordem de auras</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D30" s="19" t="inlineStr">
         <is>
           <t>Haste &gt; Physical Damage &gt; Energy Shield &gt; Heals Allies &gt; Hinder. Bônus: Always Shocks, Breaks Armour, Stuns, extra chaos/lightning ou crítico.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="49" customHeight="1">
-      <c r="A30" s="19" t="inlineStr">
+    <row r="31" ht="49" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
         <is>
           <t>Dano</t>
         </is>
       </c>
-      <c r="B30" s="23" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Catha's Balance: dano por golpe</t>
         </is>
       </c>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="D31" s="19" t="inlineStr">
         <is>
           <t>Companions ganham 60% do dano da main-hand. Compare armas pelo dano mínimo–máximo por golpe, não pelo DPS: a Chober Chaber bate devagar, mas tem o maior dano por golpe e ainda dá +Minion Skills e Spirit.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="34" customHeight="1">
-      <c r="A31" s="19" t="inlineStr">
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Dano</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Cuidado com o weapon swap</t>
         </is>
       </c>
-      <c r="D31" s="19" t="inlineStr">
+      <c r="D32" s="19" t="inlineStr">
         <is>
           <t>A Catha's Balance lê a main-hand do set ATIVO. Se trocar para um set com arma fraca, o zoo perde dano. No Atlas, fique no set da arma forte (ou coloque arma forte nos dois).</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="49" customHeight="1">
-      <c r="A32" s="19" t="inlineStr">
+    <row r="33" ht="49" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Dano</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Jeweller's no macaco primeiro</t>
         </is>
       </c>
-      <c r="D32" s="19" t="inlineStr">
+      <c r="D33" s="19" t="inlineStr">
         <is>
           <t>Todos os sockets vão para o Tame Beast do Silverfist antes de qualquer outra gem. Com o Effigy, o Azmerian Wolf passa a ser prioridade (Perfect Jeweller's se o Effigy estiver com poucos sockets — não funciona em item corrompido).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="34" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
-        <is>
-          <t>Dano</t>
-        </is>
-      </c>
-      <c r="B33" s="23" t="inlineStr">
-        <is>
-          <t>Médio</t>
-        </is>
-      </c>
-      <c r="C33" s="18" t="inlineStr">
-        <is>
-          <t>Loyalty em todos</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>Loyalty soma em todos os companions — dá para colocar até no Silverfist quando o dano já sobra e você quer mais segurança.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="34" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>Gameplay</t>
+          <t>Dano</t>
         </is>
       </c>
       <c r="B34" s="23" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Médio</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>Fique perto (Presence)</t>
+          <t>Loyalty em todos</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>Vários bônus (Shared Companion Damage, auras dos beasts) exigem companions na sua Presence. Não corra muito à frente do zoo em bosses.</t>
+          <t>Loyalty soma em todos os companions — dá para colocar até no Silverfist quando o dano já sobra e você quer mais segurança.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="34" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>Defesa</t>
+          <t>Gameplay</t>
         </is>
       </c>
       <c r="B35" s="23" t="inlineStr">
@@ -11209,12 +11209,12 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>DoT é o que mata</t>
+          <t>Fique perto (Presence)</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Evasion + Deflection seguram hits, não DoT. Leve Ruby (burn), Antidote (poison) e Staunching (bleed). Resists sempre no cap.</t>
+          <t>Vários bônus (Shared Companion Damage, auras dos beasts) exigem companions na sua Presence. Não corra muito à frente do zoo em bosses.</t>
         </is>
       </c>
     </row>
@@ -11226,71 +11226,93 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
+          <t>Fácil</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>DoT é o que mata</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>Evasion + Deflection seguram hits, não DoT. Leve Ruby (burn), Antidote (poison) e Staunching (bleed). Resists sempre no cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="inlineStr">
+        <is>
           <t>Médio</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C37" s="18" t="inlineStr">
         <is>
           <t>Idolatry x runas de resist</t>
         </is>
       </c>
-      <c r="D36" s="19" t="inlineStr">
+      <c r="D37" s="19" t="inlineStr">
         <is>
           <t>Cada Augment que não é Idol tira 4% de todas as resistências. Troque runas/soul cores de resist por Idols só depois de capar resists pelo gear.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="49" customHeight="1">
-      <c r="A37" s="19" t="inlineStr">
+    <row r="38" ht="49" customHeight="1">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Economia</t>
         </is>
       </c>
-      <c r="B37" s="23" t="inlineStr">
+      <c r="B38" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C37" s="18" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>Regex de vendor</t>
         </is>
       </c>
-      <c r="D37" s="19" t="inlineStr">
+      <c r="D38" s="19" t="inlineStr">
         <is>
           <t>Cole na busca do vendor para destacar upgrades: !regen|block|bow|mace|quarterstaff|armour:|accuracy|energy shield:""resi|\d+% i.+mov|ph.*da|\d l.+da|^\+.*ills$|^\+.*ion skills$|ck spe|o (all a|d)|evasion|spirit</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="34" customHeight="1">
-      <c r="A38" s="19" t="inlineStr">
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
         <is>
           <t>Economia</t>
         </is>
       </c>
-      <c r="B38" s="23" t="inlineStr">
+      <c r="B39" s="23" t="inlineStr">
         <is>
           <t>Fácil</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>Compre a Chober Chaber cedo</t>
         </is>
       </c>
-      <c r="D38" s="19" t="inlineStr">
+      <c r="D39" s="19" t="inlineStr">
         <is>
           <t>A Chober Chaber costuma custar poucos Exalts. Compre já Runeforged no Ato 3–4 e guarde: com a Catha's Balance ela vira a principal fonte de dano do zoo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D38"/>
+  <autoFilter ref="A3:D39"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B4:B38">
+  <conditionalFormatting sqref="B4:B39">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="5">
       <formula>"Fácil"</formula>
     </cfRule>
@@ -12535,7 +12557,7 @@
       </c>
       <c r="E13" s="42" t="inlineStr"/>
     </row>
-    <row r="14" ht="49" customHeight="1">
+    <row r="14" ht="64" customHeight="1">
       <c r="A14" s="23" t="n">
         <v>11</v>
       </c>
@@ -12551,7 +12573,7 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>O objetivo são 2–3 auras T1 (Physical/Haste &gt; ES/Invulnerability &gt; Temporal Bubble &gt; Elemental Res) em beasts de 21–25% de Spirit: Swarming Wisp, Crag Leaper, Quill/Coconut Crab.</t>
+          <t>Com Sylvan's Effigy, o objetivo são 2–3 auras T1 (antes dele só cabe 1) (Physical/Haste &gt; ES/Invulnerability &gt; Temporal Bubble &gt; Elemental Res) em beasts de 21–25% de Spirit: Swarming Wisp, Crag Leaper, Quill/Coconut Crab.</t>
         </is>
       </c>
       <c r="E14" s="42" t="inlineStr">
@@ -22709,12 +22731,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Terceiro companion, marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
+          <t>Macaco + 1 beast de aura (o limite do Trusted Kinship é 2 companions), marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3 companions + chaos</t>
+          <t>2 companions + chaos</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -25302,7 +25324,7 @@
       </c>
       <c r="D49" s="26" t="inlineStr">
         <is>
-          <t>Terceiro companion, marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
+          <t>Macaco + 1 beast de aura (o limite do Trusted Kinship é 2 companions), marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
         </is>
       </c>
       <c r="E49" s="26" t="inlineStr">
@@ -27377,7 +27399,7 @@
       </c>
       <c r="C89" s="27" t="inlineStr">
         <is>
-          <t>3 aura bots (Haste/Physical/ES).</t>
+          <t>Com Sylvan's Effigy: 3 aura bots (Haste/Physical/ES).</t>
         </is>
       </c>
       <c r="D89" s="26" t="inlineStr">
@@ -28752,7 +28774,7 @@
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="13" t="inlineStr">
         <is>
-          <t>ATO 4  ·  Nv 46–55  ·  3 companions + chaos</t>
+          <t>ATO 4  ·  Nv 46–55  ·  2 companions + chaos</t>
         </is>
       </c>
       <c r="B45" s="14" t="n"/>
@@ -28761,7 +28783,7 @@
       <c r="E45" s="14" t="n"/>
       <c r="F45" s="14" t="n"/>
     </row>
-    <row r="46" ht="19" customHeight="1">
+    <row r="46" ht="34" customHeight="1">
       <c r="A46" s="28" t="inlineStr">
         <is>
           <t>Objetivo</t>
@@ -28769,7 +28791,7 @@
       </c>
       <c r="B46" s="29" t="inlineStr">
         <is>
-          <t>Terceiro companion, marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
+          <t>Macaco + 1 beast de aura (o limite do Trusted Kinship é 2 companions), marks e curse. Entram Evergrasping Ring (aliados ganham dano de chaos) e Withering Presence (inimigos recebem mais chaos): as duas peças se multiplicam.</t>
         </is>
       </c>
       <c r="C46" s="10" t="n"/>
@@ -28865,7 +28887,7 @@
       </c>
       <c r="B52" s="29" t="inlineStr">
         <is>
-          <t>3 companions · Evergrasping Ring ×2 + Withering Presence · Testes de resistência do Ato 4 feitos</t>
+          <t>2 companions (macaco + aura) · Evergrasping Ring ×2 + Withering Presence · Testes de resistência do Ato 4 feitos</t>
         </is>
       </c>
       <c r="C52" s="10" t="n"/>
@@ -29422,7 +29444,7 @@
       </c>
       <c r="B95" s="29" t="inlineStr">
         <is>
-          <t>Giant's Blood + Chober + Effigy · Zekoa com Extra Crits/Haste · 3 aura bots · Forgotten Warden + Spirit Vessel</t>
+          <t>Giant's Blood + Chober + Effigy · Zekoa com Extra Crits/Haste · 3 aura bots (com Sylvan's Effigy) · Forgotten Warden + Spirit Vessel</t>
         </is>
       </c>
       <c r="C95" s="10" t="n"/>
@@ -31005,7 +31027,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="49" customHeight="1">
+    <row r="32" ht="79" customHeight="1">
       <c r="A32" s="26" t="inlineStr">
         <is>
           <t>Ato 4</t>
@@ -31013,7 +31035,7 @@
       </c>
       <c r="B32" s="27" t="inlineStr">
         <is>
-          <t>Tame Beast (3º beast)</t>
+          <t>Tame Beast (3º beast: só com Sylvan's Effigy)</t>
         </is>
       </c>
       <c r="C32" s="26" t="inlineStr">
@@ -31028,12 +31050,12 @@
       <c r="H32" s="26" t="inlineStr"/>
       <c r="I32" s="26" t="inlineStr">
         <is>
-          <t>Aura bot / captura</t>
+          <t>Captura / guardar para o Effigy</t>
         </is>
       </c>
       <c r="J32" s="26" t="inlineStr">
         <is>
-          <t>Só quando ganhar mais Spirit (Lythara +40 nos Interlúdios, capacete/amuleto com Spirit). Até lá, deixe a gem vazia só para capturar: Quill Crab e Coconut Crab aparecem no Whakapanu Island (Ato 4).</t>
+          <t>Com Trusted Kinship o limite é 2 companions de tipos diferentes (texto do keystone). O 3º só pode ficar ativo com o Sylvan's Effigy ("any number of Companions"). Até lá, use esta gem vazia só para capturar e guardar um Swarming Wisp / Plague Swarm com aura Physical.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige requisito do Sylvan's Effigy (nível 62) e troca a fonte de níveis para o Path of Building
O campo levelRequired do poe.ninja não é o requisito real (dizia 78; o item no jogo pede 62).
- Níveis agora vêm do Path of Building (Requires Level do unique ou do tipo base, marcado como 'confira no item')
- Remove os níveis de Runeforged/Runemastered que vinham da mesma fonte
- Effigy, Azmerian Wolf, marco e ordem de compra ajustados para o nível 62
- Forgotten Warden: skill Spirit Vessel confirmada no PoB

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
+++ b/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
@@ -14251,7 +14251,7 @@
       </c>
       <c r="J13" s="19" t="inlineStr">
         <is>
-          <t>Runeforged (nv 55) ≈ 0,04 div · Para usar com sceptre precisa de Giant's Blood (Treefingers no começo, keystone na árvore depois). Giant's Blood TRIPLICA os requisitos de atributo: resolva com The Vertex (versão 'Equipment has no Attribute Requirements').</t>
+          <t>Runeforged ≈ 0,04 div · Para usar com sceptre precisa de Giant's Blood (Treefingers no começo, keystone na árvore depois). Giant's Blood TRIPLICA os requisitos de atributo: resolva com The Vertex (versão 'Equipment has no Attribute Requirements').</t>
         </is>
       </c>
     </row>
@@ -14398,7 +14398,7 @@
       </c>
       <c r="J16" s="19" t="inlineStr">
         <is>
-          <t>Runeforged (nv 40) ≈ 0,08 div · Base custa quase nada; equipe logo depois de capturar o Silverfist.</t>
+          <t>Runeforged ≈ 0,08 div · Base custa quase nada; equipe logo depois de capturar o Silverfist.</t>
         </is>
       </c>
     </row>
@@ -15476,7 +15476,7 @@
       </c>
       <c r="J39" s="19" t="inlineStr">
         <is>
-          <t>Runeforged (nv 38) ≈ 0,003 div · Runemastered (nv 55) ≈ 0,41 div · Só considere se não usar a rota Chober Chaber.</t>
+          <t>Runeforged ≈ 0,003 div · Runemastered ≈ 0,41 div · Só considere se não usar a rota Chober Chaber.</t>
         </is>
       </c>
     </row>
@@ -26192,7 +26192,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" ht="34" customHeight="1">
+    <row r="66" ht="49" customHeight="1">
       <c r="A66" s="23" t="n">
         <v>63</v>
       </c>
@@ -26201,9 +26201,9 @@
           <t>Interlúdios</t>
         </is>
       </c>
-      <c r="C66" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C66" s="18" t="inlineStr">
+        <is>
+          <t>Sylvan's Effigy liberado (requer nível 62, ~1 div): tire o Rattling Sceptre, Skeletal Cleric vira o alvo do Pain Offering e ative mais beasts de aura conforme o Spirit.</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -26972,7 +26972,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" ht="34" customHeight="1">
+    <row r="81" ht="19" customHeight="1">
       <c r="A81" s="25" t="n">
         <v>78</v>
       </c>
@@ -26981,9 +26981,9 @@
           <t>T15+ (Effigy)</t>
         </is>
       </c>
-      <c r="C81" s="27" t="inlineStr">
-        <is>
-          <t>Sylvan's Effigy (~1 div): Azmerian Wolf, Discipline, companions ilimitados.</t>
+      <c r="C81" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="D81" s="26" t="inlineStr">
@@ -34801,7 +34801,7 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Nv 78</t>
+          <t>Nv 62+</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Corrige afirmação sobre Haste em crabs: é sorte, não é fácil
Conferido no guia de beasts do Mattjestic: crabs são onde é mais fácil achar todas as auras T1; Haste exige farmar essences. Quadrilla, Swarming Wisp, Crag Leaper e Hyena Demon não rolam Haste.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
+++ b/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
@@ -10558,7 +10558,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="34" customHeight="1">
+    <row r="6" ht="64" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Captura</t>
@@ -10576,7 +10576,7 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Beasts com a tag very_fast_movement (ex.: Crag Leaper) nunca rolam Haste Aura. Procure Haste em crabs.</t>
+          <t>Beasts com a tag very_fast_movement (ex.: Crag Leaper) nunca rolam Haste Aura. Pelo guia do Mattjestic, Quadrilla, Swarming Wisp e Hyena Demon também não. Para Haste, farme essences de crab no Whakapanu Island (Ato 4) — crabs são onde é mais fácil achar todas as auras T1, mas Haste continua sendo sorte e pode levar várias tentativas.</t>
         </is>
       </c>
     </row>
@@ -35707,7 +35707,7 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>Haste Aura (o mais fácil de achar)</t>
+          <t>Qualquer aura T1, inclusive Haste (sorte: farme essences de crab)</t>
         </is>
       </c>
       <c r="G5" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Spirit Vessel: um setup por fase e sem contradição com o card do item
- Até o nível 90: Loyalty + Furious Slam + Arctic Howl + Rapid Attacks II + Rage III (Giant's Blood Endgame do Mattjestic)
- 90+: Loyalty + Devour + Oil Barrage + Salvo + Living Lightning II
- Salvo e Living Lightning II são supports, não skills; remove os '+20%/+80% more' não confirmados
- Sockets do Forgotten Warden mostram só Idols; itens adaptados usam a versão da fase mais próxima

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
+++ b/planilha/poe2_spirit_walker_silverfist_atlas.xlsx
@@ -20771,7 +20771,7 @@
       </c>
       <c r="E224" s="19" t="inlineStr">
         <is>
-          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Spirit Vessel: Furious Slam + Arctic Howl</t>
+          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol</t>
         </is>
       </c>
     </row>
@@ -21042,7 +21042,7 @@
       </c>
       <c r="E237" s="19" t="inlineStr">
         <is>
-          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Spirit Vessel: Furious Slam + Arctic Howl</t>
+          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol</t>
         </is>
       </c>
     </row>
@@ -21668,7 +21668,7 @@
         </is>
       </c>
     </row>
-    <row r="269" ht="94" customHeight="1">
+    <row r="269" ht="79" customHeight="1">
       <c r="A269" s="19" t="inlineStr"/>
       <c r="B269" s="54" t="inlineStr">
         <is>
@@ -21687,7 +21687,7 @@
       </c>
       <c r="E269" s="19" t="inlineStr">
         <is>
-          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Spirit Vessel: Devour + Oil Barrage + Salvo + Living Lightning</t>
+          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Hawk Idol</t>
         </is>
       </c>
     </row>
@@ -22008,7 +22008,7 @@
         </is>
       </c>
     </row>
-    <row r="285" ht="94" customHeight="1">
+    <row r="285" ht="79" customHeight="1">
       <c r="A285" s="19" t="inlineStr"/>
       <c r="B285" s="54" t="inlineStr">
         <is>
@@ -22027,7 +22027,7 @@
       </c>
       <c r="E285" s="19" t="inlineStr">
         <is>
-          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Spirit Vessel: Devour + Oil Barrage + Salvo + Living Lightning</t>
+          <t>+(70-100) to Deflection Rating per 50 missing Energy Shield ; (200-271)% increased Evasion and Energy Shield ; Companions have (30-50)% increased maximum Life ; (10-15)% of Damage from Deflected Hits is taken from Damageable Companion's Life before you ; (+1 mod de ataque/utilidade que não importa para o zoo)  |  Sockets/versão: Fox Idol, Hawk Idol</t>
         </is>
       </c>
     </row>
@@ -27087,7 +27087,7 @@
       </c>
       <c r="C83" s="27" t="inlineStr">
         <is>
-          <t>Forgotten Warden: Spirit Vessel com Furious Slam + Arctic Howl.</t>
+          <t>Forgotten Warden: Spirit Vessel com Furious Slam + Arctic Howl (+ Loyalty, Rapid Attacks II, Rage III).</t>
         </is>
       </c>
       <c r="D83" s="26" t="inlineStr">
@@ -32155,7 +32155,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="34" customHeight="1">
+    <row r="60" ht="79" customHeight="1">
       <c r="A60" s="19" t="inlineStr">
         <is>
           <t>T15+ (Effigy)</t>
@@ -32198,12 +32198,12 @@
       </c>
       <c r="I60" s="19" t="inlineStr">
         <is>
-          <t>Companion grátis</t>
+          <t>Companion do Forgotten Warden</t>
         </is>
       </c>
       <c r="J60" s="19" t="inlineStr">
         <is>
-          <t>Vem do Forgotten Warden. Furious Slam (Bear) e Arctic Howl (Werewolf) socketados: +20% more dano por skill diferente.</t>
+          <t>Vem do Forgotten Warden. USE ESTE até o nível 90: é o setup "Giant's Blood Endgame" do Mattjestic — 2 gems de skill (Furious Slam de Bear e Arctic Howl de Werewolf) + Loyalty, Rapid Attacks II e Rage III. No endgame (nível 90+) ele troca para Devour + Oil Barrage + Salvo + Living Lightning II.</t>
         </is>
       </c>
     </row>
@@ -32779,7 +32779,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="19" customHeight="1">
+    <row r="73" ht="79" customHeight="1">
       <c r="A73" s="26" t="inlineStr">
         <is>
           <t>Arbiter / Min-max</t>
@@ -32822,12 +32822,12 @@
       </c>
       <c r="I73" s="26" t="inlineStr">
         <is>
-          <t>Companion grátis</t>
+          <t>Companion do Forgotten Warden</t>
         </is>
       </c>
       <c r="J73" s="26" t="inlineStr">
         <is>
-          <t>4 skills diferentes socketadas = +80% more dano do Vessel.</t>
+          <t>Setup de endgame (nível 90+) do Mattjestic, usado em todas as variantes dele de Endgame Mapping/Bossing: 2 gems de skill de Wyvern (Devour e Oil Barrage) + os supports Loyalty, Salvo e Living Lightning II. Antes do 90, use a versão com Furious Slam + Arctic Howl (fase T15).</t>
         </is>
       </c>
     </row>
@@ -33191,7 +33191,7 @@
       </c>
       <c r="C84" s="31" t="inlineStr">
         <is>
-          <t>Skill de Werewolf socketada no Spirit Vessel: congela e dá dano de frio aos aliados.</t>
+          <t>Gem de SKILL de Werewolf (não é support) socketada no Spirit Vessel. Setup T15 do Mattjestic, junto com Furious Slam.</t>
         </is>
       </c>
     </row>
@@ -33347,7 +33347,7 @@
       </c>
       <c r="C97" s="31" t="inlineStr">
         <is>
-          <t>Skill de Wyvern socketada no Spirit Vessel (versão endgame).</t>
+          <t>Gem de SKILL de Wyvern (não é support) socketada no Spirit Vessel. Setup de endgame (nível 90+) do Mattjestic.</t>
         </is>
       </c>
     </row>
@@ -33479,7 +33479,7 @@
       </c>
       <c r="C108" s="31" t="inlineStr">
         <is>
-          <t>Skill de Bear socketada no Spirit Vessel: o Vessel vira urso e dá slams. Cada skill diferente socketada = +20% more dano do Vessel.</t>
+          <t>Gem de SKILL de Bear (não é support) que vai socketada no Spirit Vessel: o Vessel passa a usar esse ataque. Setup T15 do Mattjestic.</t>
         </is>
       </c>
     </row>
@@ -33587,7 +33587,7 @@
       </c>
       <c r="C117" s="31" t="inlineStr">
         <is>
-          <t>Skill socketada no Spirit Vessel.</t>
+          <t>SUPPORT (não é skill) usado no Spirit Vessel no setup de endgame do Mattjestic, junto com Devour e Oil Barrage.</t>
         </is>
       </c>
     </row>
@@ -33767,7 +33767,7 @@
       </c>
       <c r="C132" s="31" t="inlineStr">
         <is>
-          <t>Skill de Wyvern socketada no Spirit Vessel.</t>
+          <t>Gem de SKILL de Wyvern (não é support) socketada no Spirit Vessel. Setup de endgame (nível 90+), junto com Devour.</t>
         </is>
       </c>
     </row>
@@ -33983,7 +33983,7 @@
       </c>
       <c r="C150" s="31" t="inlineStr">
         <is>
-          <t>Skill socketada no Spirit Vessel.</t>
+          <t>SUPPORT (não é skill) usado no Spirit Vessel no setup de endgame do Mattjestic, junto com Devour e Oil Barrage.</t>
         </is>
       </c>
     </row>

</xml_diff>